<commit_message>
docs(evidence): T1 and T2 checkpoint bundles; roadmap statuses; harness checkpoint log
T1 (filtered gate rows, commit 4157c74): 7 PASS, CI-001 FAIL with the root cause
note in evidence/T1/ci-root-cause.md (account-level Actions condition inferred;
repository-admin action). T2 (full run): 49 PASS, 7 operator-gated FAIL
(CI-001..004, VCS-003, VCS-004, REL-003), 2 MANUAL; MIG-001 re-measured PASS in
T2-supplement after two runner fixes (absolute interpreter path; the 2.16.0 tag
predates the golden corpus). Both gates open; M3 waits on CI and review.
roadmap.xlsx: 21 items complete, 1 in progress, 4 blocked on operator action,
11 ledger rows at independently-reproduced. harness.md gains §9 Checkpoint log.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evolution/roadmap.xlsx
+++ b/docs/evolution/roadmap.xlsx
@@ -43,7 +43,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,9 +126,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1259,9 +1251,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>complete: evidence/T1 (7 PASS; CI-001 FAIL diagnosed, operator)</t>
         </is>
       </c>
     </row>
@@ -1306,9 +1298,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>complete: evidence/T2 (49+1 PASS on 4157c74; 7 operator-gated FAIL; 2 MANUAL)</t>
         </is>
       </c>
     </row>
@@ -1353,9 +1345,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>in-progress: GOV-001…003, CON-002 PASS on the branch; CI-001/002/004 blocked on the Actions startup failure (operator); VCS-003 awaits an approving review (operator)</t>
         </is>
       </c>
     </row>
@@ -1400,9 +1392,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M3 gate)</t>
         </is>
       </c>
     </row>
@@ -1447,9 +1439,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M4 gate); PERF-002, RB-002, SEC-001 already PASS on the branch; ACC-003 needs a listener</t>
         </is>
       </c>
     </row>
@@ -1494,9 +1486,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M5 gate)</t>
         </is>
       </c>
     </row>
@@ -1839,17 +1831,17 @@
           <t>M1 observability gate</t>
         </is>
       </c>
-      <c r="Z2" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB2" s="4" t="inlineStr">
         <is>
-          <t>scripts/harness.sh; evidence/T1/summary.tsv</t>
+          <t>commit a8e8690 (+ hardening 4157c74): scripts/harness.sh; evidence/T1, T2 bundles</t>
         </is>
       </c>
       <c r="AC2" s="4" t="inlineStr">
@@ -1999,17 +1991,17 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="Z3" s="4" t="inlineStr">
-        <is>
-          <t>implemented (uncommitted)</t>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="AB3" s="4" t="inlineStr">
         <is>
-          <t>git log</t>
+          <t>commits 2f4ca49, a8e8690: docs/evolution + evidence/T0 committed</t>
         </is>
       </c>
       <c r="AC3" s="4" t="inlineStr"/>
@@ -2155,17 +2147,17 @@
           <t>M1 portability gate</t>
         </is>
       </c>
-      <c r="Z4" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>harness T1 HARNESS-PORT-001.log</t>
+          <t>commit 5a3244f; evidence/T1 HARNESS-PORT-001</t>
         </is>
       </c>
       <c r="AC4" s="4" t="inlineStr">
@@ -2315,17 +2307,17 @@
           <t>M1 (diagnosis), M3 CI gate</t>
         </is>
       </c>
-      <c r="Z5" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z5" s="4" t="inlineStr">
+        <is>
+          <t>blocked</t>
         </is>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
-          <t>gh run list; ci-root-cause.md</t>
+          <t>diagnosed: evidence/T1/ci-root-cause.md (account-level Actions condition inferred; billing unreadable with this token); repository-admin action required</t>
         </is>
       </c>
       <c r="AC5" s="4" t="inlineStr">
@@ -2475,17 +2467,17 @@
           <t>M1 data-safety gate</t>
         </is>
       </c>
-      <c r="Z6" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
-          <t>`git log origin/release/engine-3.0.0`; harness T1 summary</t>
+          <t>commits 4a75778, 2f4ca49 on release/engine-3.0.0; pushed; evidence/T1 HARNESS-VCS-001/002</t>
         </is>
       </c>
       <c r="AC6" s="4" t="inlineStr">
@@ -2635,17 +2627,17 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="Z7" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t>commit touching uv.lock; harness T1 summary</t>
+          <t>commit 5a3244f (uv.lock 3.0.0); evidence/T1 HARNESS-REL-004</t>
         </is>
       </c>
       <c r="AC7" s="4" t="inlineStr">
@@ -2795,17 +2787,17 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="Z8" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
-          <t>evidence/T2/summary.tsv</t>
+          <t>evidence/T2 HARNESS-ACC-004</t>
         </is>
       </c>
       <c r="AC8" s="4" t="inlineStr"/>
@@ -2951,17 +2943,17 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="Z9" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z9" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
-          <t>evidence/T2/HARNESS-PORT-00*.log</t>
+          <t>evidence/T2 HARNESS-PORT-001…004 (3.10/3.11/3.12 green on the branch head)</t>
         </is>
       </c>
       <c r="AC9" s="4" t="inlineStr"/>
@@ -3107,17 +3099,17 @@
           <t>M2 contract gate</t>
         </is>
       </c>
-      <c r="Z10" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
-          <t>ADR diffs</t>
+          <t>commits 09e1dfa, 4157c74; evidence/T2 HARNESS-GOV-004/006</t>
         </is>
       </c>
       <c r="AC10" s="4" t="inlineStr"/>
@@ -3263,17 +3255,17 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="Z11" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
-          <t>index.md diff</t>
+          <t>commit 09e1dfa; evidence/T2 HARNESS-GOV-005</t>
         </is>
       </c>
       <c r="AC11" s="4" t="inlineStr"/>
@@ -3419,17 +3411,17 @@
           <t>M2 (non-blocking)</t>
         </is>
       </c>
-      <c r="Z12" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
-          <t>.agent-tasks state</t>
+          <t>commit 09e1dfa; evidence/T2 HARNESS-GOV-007</t>
         </is>
       </c>
       <c r="AC12" s="4" t="inlineStr">
@@ -3579,17 +3571,17 @@
           <t>M2 contract gate</t>
         </is>
       </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z13" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
-          <t>capabilities.py diff; DIAGNOSTIC_CODES.md regenerated</t>
+          <t>commits 901191c, 4157c74 (40 registered codes); evidence/T2 HARNESS-CON-001</t>
         </is>
       </c>
       <c r="AC13" s="4" t="inlineStr">
@@ -3739,17 +3731,17 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="Z14" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
-          <t>cli.py diff</t>
+          <t>commit cd06e1c; evidence/T2 HARNESS-CON-003</t>
         </is>
       </c>
       <c r="AC14" s="4" t="inlineStr"/>
@@ -3895,17 +3887,17 @@
           <t>M2 contract gate</t>
         </is>
       </c>
-      <c r="Z15" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z15" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB15" s="4" t="inlineStr">
         <is>
-          <t>schema.py / sdk.py diff</t>
+          <t>commit aa3c9d6; evidence/T2 HARNESS-CON-004</t>
         </is>
       </c>
       <c r="AC15" s="4" t="inlineStr">
@@ -4055,7 +4047,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z16" s="7" t="inlineStr">
+      <c r="Z16" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4065,7 +4057,7 @@
       </c>
       <c r="AB16" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row A1; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row A1; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC16" s="4" t="inlineStr">
@@ -4215,7 +4207,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z17" s="7" t="inlineStr">
+      <c r="Z17" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4225,7 +4217,7 @@
       </c>
       <c r="AB17" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row A2; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row A2; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC17" s="4" t="inlineStr">
@@ -4375,7 +4367,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z18" s="7" t="inlineStr">
+      <c r="Z18" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4385,7 +4377,7 @@
       </c>
       <c r="AB18" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row A3; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row A3; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC18" s="4" t="inlineStr">
@@ -4535,7 +4527,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z19" s="7" t="inlineStr">
+      <c r="Z19" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4545,7 +4537,7 @@
       </c>
       <c r="AB19" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row A4; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row A4; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC19" s="4" t="inlineStr">
@@ -4695,7 +4687,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z20" s="7" t="inlineStr">
+      <c r="Z20" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4705,7 +4697,7 @@
       </c>
       <c r="AB20" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M1; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M1; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC20" s="4" t="inlineStr">
@@ -4855,7 +4847,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z21" s="7" t="inlineStr">
+      <c r="Z21" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -4865,7 +4857,7 @@
       </c>
       <c r="AB21" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M2; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M2; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC21" s="4" t="inlineStr">
@@ -5015,7 +5007,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z22" s="7" t="inlineStr">
+      <c r="Z22" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -5025,7 +5017,7 @@
       </c>
       <c r="AB22" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M3; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M3; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC22" s="4" t="inlineStr">
@@ -5175,7 +5167,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z23" s="7" t="inlineStr">
+      <c r="Z23" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -5185,7 +5177,7 @@
       </c>
       <c r="AB23" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M4; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M4; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC23" s="4" t="inlineStr">
@@ -5335,7 +5327,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z24" s="7" t="inlineStr">
+      <c r="Z24" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -5345,7 +5337,7 @@
       </c>
       <c r="AB24" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M5; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M5; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC24" s="4" t="inlineStr">
@@ -5495,7 +5487,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z25" s="7" t="inlineStr">
+      <c r="Z25" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -5505,7 +5497,7 @@
       </c>
       <c r="AB25" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row M6; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row M6; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC25" s="4" t="inlineStr">
@@ -5655,7 +5647,7 @@
           <t>M2 test gate; M4 migration gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z26" s="7" t="inlineStr">
+      <c r="Z26" s="6" t="inlineStr">
         <is>
           <t>independently-reproduced</t>
         </is>
@@ -5665,7 +5657,7 @@
       </c>
       <c r="AB26" s="4" t="inlineStr">
         <is>
-          <t>docs/MUSICAL_CORRECTNESS.md row G1; evidence/T0 (this assessment)</t>
+          <t>docs/MUSICAL_CORRECTNESS.md row G1; evidence/T0 (this assessment); committed as 4a75778 on release/engine-3.0.0; evidence/T2 (branch head) PASS; awaits CI (ci-verified) and tag (released)</t>
         </is>
       </c>
       <c r="AC26" s="4" t="inlineStr">
@@ -5815,17 +5807,17 @@
           <t>M3 contract gate</t>
         </is>
       </c>
-      <c r="Z27" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z27" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB27" s="4" t="inlineStr">
         <is>
-          <t>Makefile diff; tests/test_makefile_targets.py</t>
+          <t>commit 9892e60: make lock-check + floor-check; ci.yml installs uv</t>
         </is>
       </c>
       <c r="AC27" s="4" t="inlineStr"/>
@@ -5971,17 +5963,17 @@
           <t>M3 review gate</t>
         </is>
       </c>
-      <c r="Z28" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z28" s="4" t="inlineStr">
+        <is>
+          <t>in-progress</t>
         </is>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
-          <t>`gh pr view --json reviews`</t>
+          <t>PR #1 open; agent code review posted as PR comment; human approval pending (operator)</t>
         </is>
       </c>
       <c r="AC28" s="4" t="inlineStr">
@@ -6131,17 +6123,17 @@
           <t>M3 contract gate</t>
         </is>
       </c>
-      <c r="Z29" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z29" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
-          <t>docs/backlog.yml diff; governance output</t>
+          <t>commit c49c46c: BL-032..BL-035; evidence/T2 HARNESS-GOV-001</t>
         </is>
       </c>
       <c r="AC29" s="4" t="inlineStr"/>
@@ -6287,17 +6279,17 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="Z30" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z30" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB30" s="4" t="inlineStr">
         <is>
-          <t>backlog.yml diff</t>
+          <t>commit c49c46c; evidence/T2 HARNESS-GOV-002</t>
         </is>
       </c>
       <c r="AC30" s="4" t="inlineStr"/>
@@ -6443,17 +6435,17 @@
           <t>M3 contract gate; M6 release gate</t>
         </is>
       </c>
-      <c r="Z31" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z31" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB31" s="4" t="inlineStr">
         <is>
-          <t>MUSICAL_CORRECTNESS.md diff</t>
+          <t>commit baecfaa; evidence/T2 HARNESS-GOV-003 (statuses advance again at T4/T6)</t>
         </is>
       </c>
       <c r="AC31" s="4" t="inlineStr"/>
@@ -6599,17 +6591,17 @@
           <t>M3 architecture gate</t>
         </is>
       </c>
-      <c r="Z32" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z32" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB32" s="4" t="inlineStr">
         <is>
-          <t>ADR-0008; sdk.py diff</t>
+          <t>commit 52b1eac + ADR-0008; evidence/T2 HARNESS-CON-002</t>
         </is>
       </c>
       <c r="AC32" s="4" t="inlineStr"/>
@@ -6755,17 +6747,17 @@
           <t>M4 migration gate</t>
         </is>
       </c>
-      <c r="Z33" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z33" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB33" s="4" t="inlineStr">
         <is>
-          <t>CHANGELOG diff</t>
+          <t>commit 3adfeb9; evidence/T2 HARNESS-REL-002</t>
         </is>
       </c>
       <c r="AC33" s="4" t="inlineStr">
@@ -6915,9 +6907,9 @@
           <t>M4 migration gate</t>
         </is>
       </c>
-      <c r="Z34" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>blocked</t>
         </is>
       </c>
       <c r="AA34" s="4" t="n">
@@ -6925,7 +6917,7 @@
       </c>
       <c r="AB34" s="4" t="inlineStr">
         <is>
-          <t>`gh run list --branch main`; harness T4 summary</t>
+          <t>gate closed: HARNESS-CI-002 cannot pass while Actions fail at startup (operator: RM-B-002) and HARNESS-VCS-003 awaits approval</t>
         </is>
       </c>
       <c r="AC34" s="4" t="inlineStr"/>
@@ -7071,9 +7063,9 @@
           <t>M5 release gate (waivable per harness §6.3)</t>
         </is>
       </c>
-      <c r="Z35" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z35" s="4" t="inlineStr">
+        <is>
+          <t>blocked</t>
         </is>
       </c>
       <c r="AA35" s="4" t="n">
@@ -7081,7 +7073,7 @@
       </c>
       <c r="AB35" s="4" t="inlineStr">
         <is>
-          <t>evidence/T5/listening-review.json</t>
+          <t>operator: a listener must judge the seven cases (index.html in evidence/T2/work is regenerable via the runner) and export listening-review.json</t>
         </is>
       </c>
       <c r="AC35" s="4" t="inlineStr">
@@ -7231,17 +7223,17 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="Z36" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z36" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB36" s="4" t="inlineStr">
         <is>
-          <t>evidence/T5/HARNESS-RB-002.log</t>
+          <t>commit 41a153f (runbook in MIGRATION_3.md); evidence/T2 HARNESS-RB-001/002</t>
         </is>
       </c>
       <c r="AC36" s="4" t="inlineStr"/>
@@ -7387,17 +7379,17 @@
           <t>M5 performance gate</t>
         </is>
       </c>
-      <c r="Z37" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z37" s="5" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB37" s="4" t="inlineStr">
         <is>
-          <t>MIGRATION_3.md diff; tests/test_perf_budget.py</t>
+          <t>commit 41a153f; evidence/T2 HARNESS-PERF-002</t>
         </is>
       </c>
       <c r="AC37" s="4" t="inlineStr">
@@ -7547,9 +7539,9 @@
           <t>M6 release gate</t>
         </is>
       </c>
-      <c r="Z38" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="Z38" s="4" t="inlineStr">
+        <is>
+          <t>blocked</t>
         </is>
       </c>
       <c r="AA38" s="4" t="n">
@@ -7557,7 +7549,7 @@
       </c>
       <c r="AB38" s="4" t="inlineStr">
         <is>
-          <t>`git ls-remote --tags origin`; evidence/T6/summary.tsv</t>
+          <t>depends on RM-C-005 and the M5 gate (listening review or waiver)</t>
         </is>
       </c>
       <c r="AC38" s="4" t="inlineStr">
@@ -8873,9 +8865,9 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>complete: evidence/T1 (7 PASS; CI-001 FAIL diagnosed, operator)</t>
         </is>
       </c>
     </row>
@@ -8915,9 +8907,9 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>complete: evidence/T2 (49+1 PASS on 4157c74; 7 operator-gated FAIL; 2 MANUAL)</t>
         </is>
       </c>
     </row>
@@ -8957,9 +8949,9 @@
           <t>M4</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>in-progress: GOV-001…003, CON-002 PASS on the branch; CI-001/002/004 blocked on the Actions startup failure (operator); VCS-003 awaits an approving review (operator)</t>
         </is>
       </c>
     </row>
@@ -8999,9 +8991,9 @@
           <t>M5</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M3 gate)</t>
         </is>
       </c>
     </row>
@@ -9041,9 +9033,9 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M4 gate); PERF-002, RB-002, SEC-001 already PASS on the branch; ACC-003 needs a listener</t>
         </is>
       </c>
     </row>
@@ -9083,9 +9075,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>not-started</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>blocked (M5 gate)</t>
         </is>
       </c>
     </row>
@@ -9749,7 +9741,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10125,7 +10117,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10313,7 +10305,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10360,7 +10352,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10407,7 +10399,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10454,7 +10446,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10501,7 +10493,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10548,7 +10540,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10595,7 +10587,7 @@
           <t>A+M</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10642,7 +10634,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10736,7 +10728,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10783,7 +10775,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10830,7 +10822,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10877,7 +10869,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10924,7 +10916,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10971,7 +10963,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11018,7 +11010,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11065,7 +11057,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11112,7 +11104,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E43" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11159,7 +11151,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11206,7 +11198,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -11253,7 +11245,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11300,7 +11292,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11347,7 +11339,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11394,7 +11386,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -11488,7 +11480,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -11723,7 +11715,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -11817,7 +11809,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -11864,7 +11856,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E59" s="9" t="inlineStr">
+      <c r="E59" s="8" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>

</xml_diff>

<commit_message>
fix(sequencer): patterned sample layers carry no voice; roadmap statuses after review
46ef6cd moved the drum-voice lookup ahead of the sample-override check and
read track["voice"], which patterned sample layers do not have; the script-mode
instruments suite caught it in the isolated gate. Use track.get("voice").
roadmap.xlsx: RM-C-003 at 80 % (nine review defects fixed, nine deferred to
BL-036..BL-044, approval pending); RM-D-001 cites the new items.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evolution/roadmap.xlsx
+++ b/docs/evolution/roadmap.xlsx
@@ -5969,11 +5969,11 @@
         </is>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
-          <t>PR #1 open; agent code review posted as PR comment; human approval pending (operator)</t>
+          <t>PR #1: eight-pass agent code review complete; 9 reproduced defects fixed on the branch (3d19d26 intent round trip + unique layer names; e5decf6 repeat slivers, groove slot under swing, clip-aware activity; 46ef6cd shared validators, explicit fidelity, helper reuse; cd55a73 tone freq:, cutdowns not loop-gated); 9 accepted findings deferred to BL-036..BL-044; review comment on the PR; human approval pending (operator)</t>
         </is>
       </c>
       <c r="AC28" s="4" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
-          <t>commit c49c46c: BL-032..BL-035; evidence/T2 HARNESS-GOV-001</t>
+          <t>commits c49c46c (BL-032..BL-035), 2178916 (BL-036..BL-044 from the review); evidence/T2 HARNESS-GOV-001</t>
         </is>
       </c>
       <c r="AC29" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(evidence): T3 partial measurement; VCS-003 accepts an owner-written sign-off comment
GitHub refuses an approving review from the account that opened the PR, so a
one-maintainer repository can never satisfy "≥1 APPROVED review". The harness
row and runner accept a comment written by the repository owner (never by an
agent) beginning "Approved by the repository owner". The owner approved in
session on 2026-09-06; the comment is not yet posted, so VCS-003 still FAILs.
CI-001/002 FAIL: Actions still end in startup_failure with zero jobs and the
runs cannot be retried. RM-C-003 at 90 %.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evolution/roadmap.xlsx
+++ b/docs/evolution/roadmap.xlsx
@@ -5969,11 +5969,11 @@
         </is>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
-          <t>PR #1: eight-pass agent code review complete; 9 reproduced defects fixed on the branch (3d19d26 intent round trip + unique layer names; e5decf6 repeat slivers, groove slot under swing, clip-aware activity; 46ef6cd shared validators, explicit fidelity, helper reuse; cd55a73 tone freq:, cutdowns not loop-gated); 9 accepted findings deferred to BL-036..BL-044; review comment on the PR; human approval pending (operator)</t>
+          <t>PR #1: eight-pass agent code review; 9 reproduced defects fixed (3d19d26, e5decf6, 46ef6cd, cd55a73, f4f4eaf); 9 findings deferred to BL-036..BL-044; owner approved in session 2026-09-06; GitHub forbids self-approval, so the owner must post the sign-off comment ("Approved by the repository owner") on PR #1 for HARNESS-VCS-003 to pass</t>
         </is>
       </c>
       <c r="AC28" s="4" t="inlineStr">

</xml_diff>